<commit_message>
Dependent dynamic dropdown, import data from pdf, waterfall chart, combo chart
</commit_message>
<xml_diff>
--- a/12. Dependendent Dyanamic & Autoformatter for worksheets/Movie List for Create Excel Dropdown Menus.xlsx
+++ b/12. Dependendent Dyanamic & Autoformatter for worksheets/Movie List for Create Excel Dropdown Menus.xlsx
@@ -2,19 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Advance_Excel_BI\12. Dependendent Dyanamic &amp; Autoformatter for worksheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26E48E4A-9C67-454F-A0BA-34E0F909F3D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:8001_{B82A23EC-C253-4C7B-9747-4EDDF5F54D82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Movie List" sheetId="5" r:id="rId1"/>
+    <sheet name="Protected" sheetId="6" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="Categories">Table2[List of Categories]</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -31,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="69">
   <si>
     <t>Title</t>
   </si>
@@ -229,13 +233,22 @@
   </si>
   <si>
     <t>List of Categories</t>
+  </si>
+  <si>
+    <t>Sports</t>
+  </si>
+  <si>
+    <t>Cartoon</t>
+  </si>
+  <si>
+    <t>Wanted</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -251,16 +264,35 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor theme="6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -268,21 +300,119 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="6"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="6"/>
+        </left>
+        <right style="thin">
+          <color theme="6"/>
+        </right>
+        <top style="thin">
+          <color theme="6"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="0"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="6"/>
+          <bgColor theme="6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -361,6 +491,16 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0A2B2867-D6A2-4B3B-A90D-585A2BA5C19C}" name="Table2" displayName="Table2" ref="A1:A19" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2" tableBorderDxfId="1">
+  <autoFilter ref="A1:A19" xr:uid="{0A2B2867-D6A2-4B3B-A90D-585A2BA5C19C}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{C525EBE6-11C7-44A5-9214-2A62E2DEDB39}" name="List of Categories" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -650,7 +790,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CD1A21F-E471-4F64-991D-48ED45D6FB8A}">
-  <dimension ref="A1:J43"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.21875" bestFit="1" customWidth="1"/>
@@ -675,9 +816,6 @@
       <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
@@ -710,9 +848,6 @@
       <c r="D3">
         <v>1989</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>16</v>
-      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -727,25 +862,19 @@
       <c r="D4">
         <v>1995</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
       </c>
       <c r="D5">
         <v>2003</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -761,9 +890,6 @@
       <c r="D6">
         <v>2002</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -778,25 +904,19 @@
       <c r="D7">
         <v>2003</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
         <v>29</v>
       </c>
       <c r="D8">
         <v>2003</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -812,9 +932,6 @@
       <c r="D9">
         <v>1939</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>58</v>
-      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -829,9 +946,6 @@
       <c r="D10">
         <v>1989</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -846,9 +960,6 @@
       <c r="D11">
         <v>1990</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -863,9 +974,6 @@
       <c r="D12">
         <v>1986</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>21</v>
-      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -880,9 +988,6 @@
       <c r="D13">
         <v>1987</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -897,9 +1002,6 @@
       <c r="D14">
         <v>1994</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>20</v>
-      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -914,9 +1016,6 @@
       <c r="D15">
         <v>1996</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>6</v>
-      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -931,11 +1030,8 @@
       <c r="D16">
         <v>2000</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>47</v>
       </c>
@@ -948,11 +1044,8 @@
       <c r="D17">
         <v>1968</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -966,7 +1059,7 @@
         <v>1999</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -980,7 +1073,7 @@
         <v>1994</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>49</v>
       </c>
@@ -994,7 +1087,7 @@
         <v>2001</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -1008,7 +1101,7 @@
         <v>1973</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>50</v>
       </c>
@@ -1022,7 +1115,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>51</v>
       </c>
@@ -1036,7 +1129,7 @@
         <v>2001</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -1050,7 +1143,7 @@
         <v>1990</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>53</v>
       </c>
@@ -1064,7 +1157,7 @@
         <v>1993</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>54</v>
       </c>
@@ -1078,7 +1171,7 @@
         <v>1986</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>18</v>
       </c>
@@ -1092,7 +1185,7 @@
         <v>2002</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>19</v>
       </c>
@@ -1106,7 +1199,7 @@
         <v>1983</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>15</v>
       </c>
@@ -1120,7 +1213,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>55</v>
       </c>
@@ -1134,7 +1227,7 @@
         <v>2001</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>56</v>
       </c>
@@ -1148,7 +1241,7 @@
         <v>1986</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>14</v>
       </c>
@@ -1316,9 +1409,134 @@
         <v>2020</v>
       </c>
     </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B44" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B44 B46:B410" xr:uid="{AA52E174-C4B3-46AA-9A54-ED808153C07F}">
+      <formula1>Categories</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70D89107-1F9F-427B-9C9C-08285370BF82}">
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:A19"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3"/>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection insertColumns="0" insertRows="0" deleteColumns="0" deleteRows="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>